<commit_message>
adding colony as variable into permanova models
</commit_message>
<xml_diff>
--- a/OutputData/StatisticsResults/MOStats_PERMANOVA_SingleInteraction.xlsx
+++ b/OutputData/StatisticsResults/MOStats_PERMANOVA_SingleInteraction.xlsx
@@ -392,16 +392,16 @@
         <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>20</v>
+        <v>95</v>
       </c>
       <c r="C2" t="n">
-        <v>793.669547229307</v>
+        <v>1337.03528111464</v>
       </c>
       <c r="D2" t="n">
-        <v>0.408831743290929</v>
+        <v>0.738867737395643</v>
       </c>
       <c r="E2" t="n">
-        <v>7.01939278252734</v>
+        <v>3.54429227279911</v>
       </c>
       <c r="F2" t="n">
         <v>0.001</v>
@@ -412,13 +412,13 @@
         <v>7</v>
       </c>
       <c r="B3" t="n">
-        <v>203</v>
+        <v>119</v>
       </c>
       <c r="C3" t="n">
-        <v>1147.64142055561</v>
+        <v>472.537952962971</v>
       </c>
       <c r="D3" t="n">
-        <v>0.591168256709071</v>
+        <v>0.261132262604358</v>
       </c>
       <c r="E3"/>
       <c r="F3"/>
@@ -428,10 +428,10 @@
         <v>8</v>
       </c>
       <c r="B4" t="n">
-        <v>223</v>
+        <v>214</v>
       </c>
       <c r="C4" t="n">
-        <v>1941.31096778492</v>
+        <v>1809.57323407761</v>
       </c>
       <c r="D4" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
added colony, seasonality, and person as independent variables to one way and pairwise permanovas
</commit_message>
<xml_diff>
--- a/OutputData/StatisticsResults/MOStats_PERMANOVA_SingleInteraction.xlsx
+++ b/OutputData/StatisticsResults/MOStats_PERMANOVA_SingleInteraction.xlsx
@@ -392,16 +392,16 @@
         <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="C2" t="n">
-        <v>1337.03528111464</v>
+        <v>1369.43303308727</v>
       </c>
       <c r="D2" t="n">
-        <v>0.738867737395643</v>
+        <v>0.756771269213266</v>
       </c>
       <c r="E2" t="n">
-        <v>3.54429227279911</v>
+        <v>3.11135640417747</v>
       </c>
       <c r="F2" t="n">
         <v>0.001</v>
@@ -412,13 +412,13 @@
         <v>7</v>
       </c>
       <c r="B3" t="n">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="C3" t="n">
-        <v>472.537952962971</v>
+        <v>440.140200990344</v>
       </c>
       <c r="D3" t="n">
-        <v>0.261132262604358</v>
+        <v>0.243228730786735</v>
       </c>
       <c r="E3"/>
       <c r="F3"/>

</xml_diff>